<commit_message>
Richiesta di Accreditamento YooMultimedia PSS 1.4 -> 1.5 - Add testcase 476
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#YOOMULTIMEDIAX1/YOO-Multimedia-SRL/YOOMULTIMEDIA-FSE-GATEWAY/1.1.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#YOOMULTIMEDIAX1/YOO-Multimedia-SRL/YOOMULTIMEDIA-FSE-GATEWAY/1.1.0/report-checklist.xlsx
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="112">
   <si>
     <t xml:space="preserve">COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -205,7 +205,7 @@
     <t xml:space="preserve">subject_application_vendor: YOO Multimedia SRL</t>
   </si>
   <si>
-    <t xml:space="preserve">subject_application_version: 1.0.0</t>
+    <t xml:space="preserve">subject_application_version: 1.1.0</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -318,6 +318,22 @@
   </si>
   <si>
     <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.a9f4347f79cf3e1cf2ff4d79eaf6d0cf8d4a82cf3fb4e942adcc54e7fc27772e.c7955e2469^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VALIDAZIONE_CDA2_PSS_CT3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-09T13:42:58Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92a0d9fa1ee781154fd41ff9bc8018a8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.a9f4347f79cf3e1cf2ff4d79eaf6d0cf8d4a82cf3fb4e942adcc54e7fc27772e.abe0342557^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t xml:space="preserve">Razionale di Applicabilità</t>
@@ -754,7 +770,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -904,6 +920,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2764,7 +2784,7 @@
       <c r="G11" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="H11" s="37" t="s">
+      <c r="H11" s="32" t="s">
         <v>58</v>
       </c>
       <c r="I11" s="33" t="s">
@@ -2787,25 +2807,50 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
-      <c r="J12" s="14"/>
-      <c r="K12" s="14"/>
-      <c r="L12" s="14"/>
-      <c r="M12" s="14"/>
-      <c r="N12" s="14"/>
-      <c r="O12" s="14"/>
-      <c r="P12" s="14"/>
-      <c r="Q12" s="14"/>
-      <c r="R12" s="14"/>
-      <c r="S12" s="14"/>
-      <c r="T12" s="14"/>
-      <c r="U12" s="15"/>
-      <c r="V12" s="3"/>
-      <c r="W12" s="16"/>
+    <row r="12" customFormat="false" ht="69.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="28" t="n">
+        <v>476</v>
+      </c>
+      <c r="B12" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="28" t="s">
+        <v>60</v>
+      </c>
+      <c r="E12" s="30" t="s">
+        <v>61</v>
+      </c>
+      <c r="F12" s="31" t="n">
+        <v>46090</v>
+      </c>
+      <c r="G12" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="H12" s="37" t="s">
+        <v>63</v>
+      </c>
+      <c r="I12" s="38" t="s">
+        <v>64</v>
+      </c>
+      <c r="J12" s="34"/>
+      <c r="K12" s="34"/>
+      <c r="L12" s="34"/>
+      <c r="M12" s="34"/>
+      <c r="N12" s="34"/>
+      <c r="O12" s="34"/>
+      <c r="P12" s="34"/>
+      <c r="Q12" s="34"/>
+      <c r="R12" s="34"/>
+      <c r="S12" s="34"/>
+      <c r="T12" s="34"/>
+      <c r="U12" s="35"/>
+      <c r="V12" s="36"/>
+      <c r="W12" s="34" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F13" s="13"/>
@@ -6875,15 +6920,15 @@
     <mergeCell ref="A6:B6"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J10:J11 M10:N11 P10:R11" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J10:J12 M10:N12 P10:R12" type="list">
       <formula1>Sheet1!$B$2:$B$3</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="T10:T11" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="T10:T12" type="list">
       <formula1>Sheet1!$A$2:$A$3</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="K10:K11" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="K10:K12" type="list">
       <formula1>'LISTA VALORI'!$A$2:$A$8</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -6909,43 +6954,43 @@
   <sheetFormatPr defaultColWidth="8.515625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="38" t="s">
-        <v>60</v>
+      <c r="A1" s="39" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="38" t="s">
-        <v>61</v>
+      <c r="A2" s="39" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="38" t="s">
-        <v>62</v>
+      <c r="A3" s="39" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="38" t="s">
-        <v>63</v>
+      <c r="A4" s="39" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="38" t="s">
-        <v>64</v>
+      <c r="A5" s="39" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="38" t="s">
-        <v>65</v>
+      <c r="A6" s="39" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="38" t="s">
-        <v>66</v>
+      <c r="A7" s="39" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="38" t="s">
-        <v>67</v>
+      <c r="A8" s="39" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -6977,170 +7022,170 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="39" t="s">
-        <v>68</v>
-      </c>
-      <c r="B1" s="40" t="s">
+      <c r="A1" s="40" t="s">
+        <v>73</v>
+      </c>
+      <c r="B1" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="40" t="s">
-        <v>69</v>
-      </c>
-      <c r="D1" s="40" t="s">
-        <v>70</v>
-      </c>
-      <c r="F1" s="41" t="s">
-        <v>71</v>
-      </c>
-      <c r="G1" s="42" t="s">
-        <v>72</v>
+      <c r="C1" s="41" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1" s="41" t="s">
+        <v>75</v>
+      </c>
+      <c r="F1" s="42" t="s">
+        <v>76</v>
+      </c>
+      <c r="G1" s="43" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="43" t="s">
-        <v>73</v>
-      </c>
-      <c r="B2" s="43" t="s">
-        <v>74</v>
-      </c>
-      <c r="C2" s="44" t="s">
-        <v>75</v>
-      </c>
-      <c r="D2" s="45" t="s">
-        <v>76</v>
+      <c r="A2" s="44" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="44" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="45" t="s">
+        <v>80</v>
+      </c>
+      <c r="D2" s="46" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="43" t="s">
-        <v>77</v>
-      </c>
-      <c r="B3" s="43" t="s">
-        <v>74</v>
-      </c>
-      <c r="C3" s="44" t="s">
-        <v>78</v>
-      </c>
-      <c r="D3" s="45" t="s">
+      <c r="A3" s="44" t="s">
+        <v>82</v>
+      </c>
+      <c r="B3" s="44" t="s">
         <v>79</v>
       </c>
+      <c r="C3" s="45" t="s">
+        <v>83</v>
+      </c>
+      <c r="D3" s="46" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="43" t="s">
-        <v>80</v>
-      </c>
-      <c r="B4" s="43" t="s">
-        <v>74</v>
-      </c>
-      <c r="C4" s="44" t="s">
-        <v>81</v>
-      </c>
-      <c r="D4" s="46" t="s">
-        <v>82</v>
+      <c r="A4" s="44" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="44" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" s="45" t="s">
+        <v>86</v>
+      </c>
+      <c r="D4" s="47" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="43" t="s">
-        <v>83</v>
-      </c>
-      <c r="B5" s="43" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="44" t="s">
-        <v>84</v>
-      </c>
-      <c r="D5" s="45" t="s">
-        <v>85</v>
+      <c r="A5" s="44" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="44" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="45" t="s">
+        <v>89</v>
+      </c>
+      <c r="D5" s="46" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="43" t="s">
-        <v>86</v>
-      </c>
-      <c r="B6" s="43" t="s">
-        <v>74</v>
-      </c>
-      <c r="C6" s="44" t="s">
-        <v>87</v>
-      </c>
-      <c r="D6" s="46" t="s">
-        <v>88</v>
+      <c r="A6" s="44" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="44" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" s="45" t="s">
+        <v>92</v>
+      </c>
+      <c r="D6" s="47" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="43" t="s">
-        <v>89</v>
-      </c>
-      <c r="B7" s="43" t="s">
-        <v>74</v>
-      </c>
-      <c r="C7" s="44" t="s">
-        <v>90</v>
-      </c>
-      <c r="D7" s="46" t="s">
-        <v>91</v>
+      <c r="A7" s="44" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" s="44" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="45" t="s">
+        <v>95</v>
+      </c>
+      <c r="D7" s="47" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="43" t="s">
-        <v>92</v>
-      </c>
-      <c r="B8" s="43" t="s">
-        <v>74</v>
-      </c>
-      <c r="C8" s="44" t="s">
-        <v>93</v>
-      </c>
-      <c r="D8" s="46" t="s">
-        <v>94</v>
+      <c r="A8" s="44" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" s="44" t="s">
+        <v>79</v>
+      </c>
+      <c r="C8" s="45" t="s">
+        <v>98</v>
+      </c>
+      <c r="D8" s="47" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="43" t="s">
+      <c r="A9" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="43" t="s">
-        <v>74</v>
-      </c>
-      <c r="C9" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="D9" s="46" t="s">
-        <v>96</v>
+      <c r="B9" s="44" t="s">
+        <v>79</v>
+      </c>
+      <c r="C9" s="45" t="s">
+        <v>100</v>
+      </c>
+      <c r="D9" s="47" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="43" t="s">
-        <v>97</v>
-      </c>
-      <c r="B10" s="43" t="s">
-        <v>74</v>
-      </c>
-      <c r="C10" s="47" t="s">
-        <v>98</v>
-      </c>
-      <c r="D10" s="45" t="s">
-        <v>99</v>
+      <c r="A10" s="44" t="s">
+        <v>102</v>
+      </c>
+      <c r="B10" s="44" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" s="48" t="s">
+        <v>103</v>
+      </c>
+      <c r="D10" s="46" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="43" t="s">
-        <v>100</v>
-      </c>
-      <c r="B11" s="43" t="s">
-        <v>74</v>
-      </c>
-      <c r="C11" s="44" t="s">
-        <v>101</v>
-      </c>
-      <c r="D11" s="46" t="s">
-        <v>102</v>
+      <c r="A11" s="44" t="s">
+        <v>105</v>
+      </c>
+      <c r="B11" s="44" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11" s="45" t="s">
+        <v>106</v>
+      </c>
+      <c r="D11" s="47" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D12" s="48"/>
+      <c r="D12" s="49"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D13" s="48"/>
+      <c r="D13" s="49"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -8125,18 +8170,18 @@
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Updated version 1.0.0 -> 1.1.0
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#YOOMULTIMEDIAX1/YOO-Multimedia-SRL/YOOMULTIMEDIA-FSE-GATEWAY/1.1.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#YOOMULTIMEDIAX1/YOO-Multimedia-SRL/YOOMULTIMEDIA-FSE-GATEWAY/1.1.0/report-checklist.xlsx
@@ -363,13 +363,13 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-09T13:42:58Z</t>
-  </si>
-  <si>
-    <t xml:space="preserve">92a0d9fa1ee781154fd41ff9bc8018a8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.a9f4347f79cf3e1cf2ff4d79eaf6d0cf8d4a82cf3fb4e942adcc54e7fc27772e.abe0342557^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t xml:space="preserve">2026-04-11T10:48:45Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">352798b3b54381aa6df1ce1ad3a72bfe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.a9f4347f79cf3e1cf2ff4d79eaf6d0cf8d4a82cf3fb4e942adcc54e7fc27772e.bda8782e7d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t xml:space="preserve">VALIDAZIONE_CDA2_PSS_CT23</t>
@@ -571,7 +571,7 @@
     <numFmt numFmtId="166" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="167" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -667,6 +667,12 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -870,7 +876,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1019,6 +1025,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1035,7 +1049,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3597,15 +3611,15 @@
         <v>74</v>
       </c>
       <c r="F29" s="31" t="n">
-        <v>46090</v>
+        <v>46123</v>
       </c>
       <c r="G29" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="H29" s="32" t="s">
+      <c r="H29" s="37" t="s">
         <v>76</v>
       </c>
-      <c r="I29" s="33" t="s">
+      <c r="I29" s="38" t="s">
         <v>77</v>
       </c>
       <c r="J29" s="34" t="s">
@@ -7809,42 +7823,42 @@
   <sheetFormatPr defaultColWidth="8.515625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="39" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="39" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="37" t="s">
+      <c r="A3" s="39" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="39" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="39" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="39" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="39" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="37" t="s">
+      <c r="A8" s="39" t="s">
         <v>86</v>
       </c>
     </row>
@@ -7877,246 +7891,246 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="40" t="s">
         <v>87</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="39" t="s">
+      <c r="C1" s="41" t="s">
         <v>88</v>
       </c>
-      <c r="D1" s="40" t="s">
+      <c r="D1" s="42" t="s">
         <v>89</v>
       </c>
-      <c r="F1" s="41" t="s">
+      <c r="F1" s="43" t="s">
         <v>90</v>
       </c>
-      <c r="G1" s="42" t="s">
+      <c r="G1" s="44" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="C2" s="44" t="s">
+      <c r="C2" s="46" t="s">
         <v>94</v>
       </c>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="47" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="45" t="s">
         <v>96</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="C3" s="44" t="s">
+      <c r="C3" s="46" t="s">
         <v>97</v>
       </c>
-      <c r="D3" s="45" t="s">
+      <c r="D3" s="47" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="45" t="s">
         <v>99</v>
       </c>
-      <c r="B4" s="43" t="s">
+      <c r="B4" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="C4" s="44" t="s">
+      <c r="C4" s="46" t="s">
         <v>100</v>
       </c>
-      <c r="D4" s="46" t="s">
+      <c r="D4" s="48" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="45" t="s">
         <v>102</v>
       </c>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="D5" s="45" t="s">
+      <c r="D5" s="47" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="45" t="s">
         <v>105</v>
       </c>
-      <c r="B6" s="43" t="s">
+      <c r="B6" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="C6" s="44" t="s">
+      <c r="C6" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="D6" s="46" t="s">
+      <c r="D6" s="48" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="45" t="s">
         <v>108</v>
       </c>
-      <c r="B7" s="43" t="s">
+      <c r="B7" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="C7" s="44" t="s">
+      <c r="C7" s="46" t="s">
         <v>109</v>
       </c>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="48" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="43" t="s">
+      <c r="A8" s="45" t="s">
         <v>111</v>
       </c>
-      <c r="B8" s="43" t="s">
+      <c r="B8" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="C8" s="46" t="s">
         <v>112</v>
       </c>
-      <c r="D8" s="46" t="s">
+      <c r="D8" s="48" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="22.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="43" t="s">
+      <c r="A9" s="45" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="43" t="s">
+      <c r="B9" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="C9" s="44" t="s">
+      <c r="C9" s="46" t="s">
         <v>114</v>
       </c>
-      <c r="D9" s="46" t="s">
+      <c r="D9" s="48" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="43" t="s">
+      <c r="A10" s="45" t="s">
         <v>116</v>
       </c>
-      <c r="B10" s="43" t="s">
+      <c r="B10" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="C10" s="47" t="s">
+      <c r="C10" s="49" t="s">
         <v>117</v>
       </c>
-      <c r="D10" s="45" t="s">
+      <c r="D10" s="47" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="43" t="s">
+      <c r="A11" s="45" t="s">
         <v>119</v>
       </c>
-      <c r="B11" s="43" t="s">
+      <c r="B11" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="C11" s="44" t="s">
+      <c r="C11" s="46" t="s">
         <v>120</v>
       </c>
-      <c r="D11" s="46" t="s">
+      <c r="D11" s="48" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="45" t="s">
         <v>122</v>
       </c>
-      <c r="B12" s="43" t="s">
+      <c r="B12" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="C12" s="44" t="s">
+      <c r="C12" s="46" t="s">
         <v>123</v>
       </c>
-      <c r="D12" s="46" t="s">
+      <c r="D12" s="48" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="43" t="s">
+      <c r="A13" s="45" t="s">
         <v>125</v>
       </c>
-      <c r="B13" s="43" t="s">
+      <c r="B13" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="C13" s="44" t="s">
+      <c r="C13" s="46" t="s">
         <v>126</v>
       </c>
-      <c r="D13" s="46" t="s">
+      <c r="D13" s="48" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="43" t="s">
+      <c r="A14" s="45" t="s">
         <v>128</v>
       </c>
-      <c r="B14" s="43" t="s">
+      <c r="B14" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="C14" s="44" t="s">
+      <c r="C14" s="46" t="s">
         <v>129</v>
       </c>
-      <c r="D14" s="46" t="s">
+      <c r="D14" s="48" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="43" t="s">
+      <c r="A15" s="45" t="s">
         <v>131</v>
       </c>
-      <c r="B15" s="43" t="s">
+      <c r="B15" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="C15" s="44" t="n">
+      <c r="C15" s="46" t="n">
         <v>521</v>
       </c>
-      <c r="D15" s="46" t="s">
+      <c r="D15" s="48" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="48" t="s">
+      <c r="A16" s="50" t="s">
         <v>133</v>
       </c>
-      <c r="B16" s="43" t="s">
+      <c r="B16" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="C16" s="49" t="s">
+      <c r="C16" s="51" t="s">
         <v>134</v>
       </c>
-      <c r="D16" s="46" t="s">
+      <c r="D16" s="48" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="43" t="s">
+      <c r="A17" s="45" t="s">
         <v>136</v>
       </c>
-      <c r="B17" s="50" t="s">
+      <c r="B17" s="52" t="s">
         <v>93</v>
       </c>
-      <c r="C17" s="51" t="s">
+      <c r="C17" s="53" t="s">
         <v>137</v>
       </c>
-      <c r="D17" s="46" t="s">
+      <c r="D17" s="48" t="s">
         <v>138</v>
       </c>
     </row>

</xml_diff>